<commit_message>
batches: rule f hull refs from igu pdfs, batch 8 drops 10 unbacked vessel type refs, review logs + decisions
</commit_message>
<xml_diff>
--- a/batches/2026-09-17_0505ET_ref_fill_rule_f/lng_carrier_backend_ref_fill.xlsx
+++ b/batches/2026-09-17_0505ET_ref_fill_rule_f/lng_carrier_backend_ref_fill.xlsx
@@ -43,7 +43,7 @@
       <sz val="12"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -63,6 +63,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFEB9C"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
   </fills>
@@ -92,7 +97,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -105,6 +110,9 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -506,7 +514,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>QA log entries: 67</t>
+          <t>QA log entries: 72</t>
         </is>
       </c>
     </row>
@@ -625,7 +633,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AT9"/>
+  <dimension ref="A1:AW9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -667,13 +675,16 @@
     <col width="15" customWidth="1" min="37" max="37"/>
     <col width="50" customWidth="1" min="38" max="38"/>
     <col width="15" customWidth="1" min="39" max="39"/>
-    <col width="25" customWidth="1" min="40" max="40"/>
+    <col width="15" customWidth="1" min="40" max="40"/>
     <col width="50" customWidth="1" min="41" max="41"/>
     <col width="15" customWidth="1" min="42" max="42"/>
-    <col width="50" customWidth="1" min="43" max="43"/>
-    <col width="15" customWidth="1" min="44" max="44"/>
+    <col width="25" customWidth="1" min="43" max="43"/>
+    <col width="50" customWidth="1" min="44" max="44"/>
     <col width="15" customWidth="1" min="45" max="45"/>
     <col width="50" customWidth="1" min="46" max="46"/>
+    <col width="15" customWidth="1" min="47" max="47"/>
+    <col width="15" customWidth="1" min="48" max="48"/>
+    <col width="50" customWidth="1" min="49" max="49"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -869,40 +880,55 @@
       </c>
       <c r="AM1" s="3" t="inlineStr">
         <is>
+          <t>Delivery delayed</t>
+        </is>
+      </c>
+      <c r="AN1" s="3" t="inlineStr">
+        <is>
+          <t>Previous delivery year(s)</t>
+        </is>
+      </c>
+      <c r="AO1" s="3" t="inlineStr">
+        <is>
+          <t>Previous delivery year(s) [ref]</t>
+        </is>
+      </c>
+      <c r="AP1" s="3" t="inlineStr">
+        <is>
           <t>[Original source]</t>
         </is>
       </c>
-      <c r="AN1" s="3" t="inlineStr">
+      <c r="AQ1" s="3" t="inlineStr">
         <is>
           <t>Operator/charterer</t>
         </is>
       </c>
-      <c r="AO1" s="3" t="inlineStr">
+      <c r="AR1" s="3" t="inlineStr">
         <is>
           <t>Operator/charterer [ref]</t>
         </is>
       </c>
-      <c r="AP1" s="3" t="inlineStr">
+      <c r="AS1" s="3" t="inlineStr">
         <is>
           <t>Contract date</t>
         </is>
       </c>
-      <c r="AQ1" s="3" t="inlineStr">
+      <c r="AT1" s="3" t="inlineStr">
         <is>
           <t>Contract date [ref]</t>
         </is>
       </c>
-      <c r="AR1" s="3" t="inlineStr">
+      <c r="AU1" s="3" t="inlineStr">
         <is>
           <t>Price</t>
         </is>
       </c>
-      <c r="AS1" s="3" t="inlineStr">
+      <c r="AV1" s="3" t="inlineStr">
         <is>
           <t>Price currency</t>
         </is>
       </c>
-      <c r="AT1" s="3" t="inlineStr">
+      <c r="AW1" s="3" t="inlineStr">
         <is>
           <t>Price [ref]</t>
         </is>
@@ -921,7 +947,7 @@
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>https://www.shipvault.com/ships/73086</t>
+          <t>https://www.shipvault.com/ships/73086, https://shipvaultapi-gjb8c.ondigitalocean.app/api/units/73086</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -1055,18 +1081,21 @@
           <t>https://www.shipvault.com/ships/73086</t>
         </is>
       </c>
-      <c r="AM2" s="2" t="inlineStr">
-        <is>
-          <t>Clarkson</t>
-        </is>
-      </c>
+      <c r="AM2" s="2" t="inlineStr"/>
       <c r="AN2" s="2" t="inlineStr"/>
       <c r="AO2" s="2" t="inlineStr"/>
-      <c r="AP2" s="2" t="inlineStr"/>
+      <c r="AP2" s="2" t="inlineStr">
+        <is>
+          <t>Clarkson</t>
+        </is>
+      </c>
       <c r="AQ2" s="2" t="inlineStr"/>
       <c r="AR2" s="2" t="inlineStr"/>
       <c r="AS2" s="2" t="inlineStr"/>
       <c r="AT2" s="2" t="inlineStr"/>
+      <c r="AU2" s="2" t="inlineStr"/>
+      <c r="AV2" s="2" t="inlineStr"/>
+      <c r="AW2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1215,26 +1244,29 @@
           <t>https://www.shipvault.com/ships/73085</t>
         </is>
       </c>
-      <c r="AM3" s="2" t="inlineStr">
-        <is>
-          <t>Clarkson</t>
-        </is>
-      </c>
+      <c r="AM3" s="2" t="inlineStr"/>
       <c r="AN3" s="2" t="inlineStr"/>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
         <is>
+          <t>Clarkson</t>
+        </is>
+      </c>
+      <c r="AQ3" s="2" t="inlineStr"/>
+      <c r="AR3" s="2" t="inlineStr"/>
+      <c r="AS3" s="2" t="inlineStr">
+        <is>
           <t>1-Sep-1976</t>
         </is>
       </c>
-      <c r="AQ3" s="4" t="inlineStr">
+      <c r="AT3" s="4" t="inlineStr">
         <is>
           <t>https://www.shipvault.com/ships/73085</t>
         </is>
       </c>
-      <c r="AR3" s="2" t="inlineStr"/>
-      <c r="AS3" s="2" t="inlineStr"/>
-      <c r="AT3" s="2" t="inlineStr"/>
+      <c r="AU3" s="2" t="inlineStr"/>
+      <c r="AV3" s="2" t="inlineStr"/>
+      <c r="AW3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -1371,10 +1403,14 @@
       <c r="AF4" s="2" t="inlineStr"/>
       <c r="AG4" s="2" t="inlineStr">
         <is>
-          <t>conventional</t>
-        </is>
-      </c>
-      <c r="AH4" s="2" t="inlineStr"/>
+          <t>FSU</t>
+        </is>
+      </c>
+      <c r="AH4" s="4" t="inlineStr">
+        <is>
+          <t>https://www.miscgroup.com/media/media-releases/misc-partners-with-pengerang-lng-two-sdn-bhd-for-lng-floating-storage-unit-project-d7503fdd178dc071ee535d98beb9e62e, https://www.insage.com.my/BursaNews/Attachment/202604/20260414/MISC-AN20260414A1-2.pdf</t>
+        </is>
+      </c>
       <c r="AI4" s="2" t="inlineStr"/>
       <c r="AJ4" s="2" t="inlineStr"/>
       <c r="AK4" s="2" t="inlineStr">
@@ -1387,34 +1423,37 @@
           <t>https://www.shipvault.com/ships/113754</t>
         </is>
       </c>
-      <c r="AM4" s="2" t="inlineStr">
-        <is>
-          <t>Clarkson</t>
-        </is>
-      </c>
+      <c r="AM4" s="2" t="inlineStr"/>
       <c r="AN4" s="2" t="inlineStr"/>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
         <is>
+          <t>Clarkson</t>
+        </is>
+      </c>
+      <c r="AQ4" s="2" t="inlineStr"/>
+      <c r="AR4" s="2" t="inlineStr"/>
+      <c r="AS4" s="2" t="inlineStr">
+        <is>
           <t>1-Apr-1999</t>
         </is>
       </c>
-      <c r="AQ4" s="4" t="inlineStr">
+      <c r="AT4" s="4" t="inlineStr">
         <is>
           <t>https://www.shipvault.com/ships/113754</t>
         </is>
       </c>
-      <c r="AR4" s="2" t="inlineStr">
-        <is>
-          <t>165</t>
-        </is>
-      </c>
-      <c r="AS4" s="2" t="inlineStr">
-        <is>
-          <t>$m</t>
-        </is>
-      </c>
-      <c r="AT4" s="4" t="inlineStr">
+      <c r="AU4" s="2" t="inlineStr">
+        <is>
+          <t>165000000.00</t>
+        </is>
+      </c>
+      <c r="AV4" s="2" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="AW4" s="4" t="inlineStr">
         <is>
           <t>https://www.shipvault.com/ships/113754</t>
         </is>
@@ -1571,34 +1610,37 @@
           <t>https://www.shipvault.com/ships/373877</t>
         </is>
       </c>
-      <c r="AM5" s="2" t="inlineStr">
-        <is>
-          <t>Clarkson</t>
-        </is>
-      </c>
+      <c r="AM5" s="2" t="inlineStr"/>
       <c r="AN5" s="2" t="inlineStr"/>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
         <is>
+          <t>Clarkson</t>
+        </is>
+      </c>
+      <c r="AQ5" s="2" t="inlineStr"/>
+      <c r="AR5" s="2" t="inlineStr"/>
+      <c r="AS5" s="2" t="inlineStr">
+        <is>
           <t>1-Nov-2014</t>
         </is>
       </c>
-      <c r="AQ5" s="4" t="inlineStr">
+      <c r="AT5" s="4" t="inlineStr">
         <is>
           <t>https://www.shipvault.com/ships/373877</t>
         </is>
       </c>
-      <c r="AR5" s="2" t="inlineStr">
-        <is>
-          <t>207</t>
-        </is>
-      </c>
-      <c r="AS5" s="2" t="inlineStr">
-        <is>
-          <t>$m</t>
-        </is>
-      </c>
-      <c r="AT5" s="4" t="inlineStr">
+      <c r="AU5" s="2" t="inlineStr">
+        <is>
+          <t>207000000.00</t>
+        </is>
+      </c>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="AW5" s="4" t="inlineStr">
         <is>
           <t>https://www.shipvault.com/ships/373877</t>
         </is>
@@ -1755,34 +1797,37 @@
           <t>https://www.shipvault.com/ships/373876</t>
         </is>
       </c>
-      <c r="AM6" s="2" t="inlineStr">
-        <is>
-          <t>Clarkson</t>
-        </is>
-      </c>
+      <c r="AM6" s="2" t="inlineStr"/>
       <c r="AN6" s="2" t="inlineStr"/>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
         <is>
+          <t>Clarkson</t>
+        </is>
+      </c>
+      <c r="AQ6" s="2" t="inlineStr"/>
+      <c r="AR6" s="2" t="inlineStr"/>
+      <c r="AS6" s="2" t="inlineStr">
+        <is>
           <t>9-Mar-2014</t>
         </is>
       </c>
-      <c r="AQ6" s="4" t="inlineStr">
+      <c r="AT6" s="4" t="inlineStr">
         <is>
           <t>https://www.shipvault.com/ships/373876</t>
         </is>
       </c>
-      <c r="AR6" s="2" t="inlineStr">
-        <is>
-          <t>207</t>
-        </is>
-      </c>
-      <c r="AS6" s="2" t="inlineStr">
-        <is>
-          <t>$m</t>
-        </is>
-      </c>
-      <c r="AT6" s="4" t="inlineStr">
+      <c r="AU6" s="2" t="inlineStr">
+        <is>
+          <t>207000000.00</t>
+        </is>
+      </c>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="AW6" s="4" t="inlineStr">
         <is>
           <t>https://www.shipvault.com/ships/373876</t>
         </is>
@@ -1822,9 +1867,9 @@
           <t>Hull 2651 (SHI)</t>
         </is>
       </c>
-      <c r="J7" s="5" t="inlineStr">
-        <is>
-          <t>https://www.shipvault.com/ships/450944, https://shipvaultapi-gjb8c.ondigitalocean.app/api/units/450944</t>
+      <c r="J7" s="6" t="inlineStr">
+        <is>
+          <t>https://www.shipvault.com/ships/450944, https://shipvaultapi-gjb8c.ondigitalocean.app/api/units/450944, https://www.datocms-assets.com/146580/1763396210-1747916410-igu-world-lng-report-2025.pdf, https://www.datocms-assets.com/146580/1783403747-igu-world-lng-report-2026.pdf</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
@@ -1943,18 +1988,21 @@
           <t>https://www.igu.org/igu-reports/2025-world-lng-report</t>
         </is>
       </c>
-      <c r="AM7" s="2" t="inlineStr">
-        <is>
-          <t>IGU</t>
-        </is>
-      </c>
+      <c r="AM7" s="2" t="inlineStr"/>
       <c r="AN7" s="2" t="inlineStr"/>
       <c r="AO7" s="2" t="inlineStr"/>
-      <c r="AP7" s="2" t="inlineStr"/>
+      <c r="AP7" s="2" t="inlineStr">
+        <is>
+          <t>IGU</t>
+        </is>
+      </c>
       <c r="AQ7" s="2" t="inlineStr"/>
       <c r="AR7" s="2" t="inlineStr"/>
       <c r="AS7" s="2" t="inlineStr"/>
       <c r="AT7" s="2" t="inlineStr"/>
+      <c r="AU7" s="2" t="inlineStr"/>
+      <c r="AV7" s="2" t="inlineStr"/>
+      <c r="AW7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -1990,9 +2038,9 @@
           <t>Hull 8102 (HDHHI)</t>
         </is>
       </c>
-      <c r="J8" s="5" t="inlineStr">
-        <is>
-          <t>https://www.shipvault.com/ships/448545</t>
+      <c r="J8" s="6" t="inlineStr">
+        <is>
+          <t>https://www.shipvault.com/ships/448545, https://www.datocms-assets.com/146580/1763396210-1747916410-igu-world-lng-report-2025.pdf, https://www.datocms-assets.com/146580/1783403747-igu-world-lng-report-2026.pdf</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
@@ -2111,18 +2159,21 @@
           <t>https://www.igu.org/igu-reports/2025-world-lng-report</t>
         </is>
       </c>
-      <c r="AM8" s="2" t="inlineStr">
-        <is>
-          <t>IGU</t>
-        </is>
-      </c>
+      <c r="AM8" s="2" t="inlineStr"/>
       <c r="AN8" s="2" t="inlineStr"/>
       <c r="AO8" s="2" t="inlineStr"/>
-      <c r="AP8" s="2" t="inlineStr"/>
+      <c r="AP8" s="2" t="inlineStr">
+        <is>
+          <t>IGU</t>
+        </is>
+      </c>
       <c r="AQ8" s="2" t="inlineStr"/>
       <c r="AR8" s="2" t="inlineStr"/>
       <c r="AS8" s="2" t="inlineStr"/>
       <c r="AT8" s="2" t="inlineStr"/>
+      <c r="AU8" s="2" t="inlineStr"/>
+      <c r="AV8" s="2" t="inlineStr"/>
+      <c r="AW8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -2158,9 +2209,9 @@
           <t>Hull 8181 (HDHHI)</t>
         </is>
       </c>
-      <c r="J9" s="5" t="inlineStr">
-        <is>
-          <t>https://www.shipvault.com/ships/461187, https://shipvaultapi-gjb8c.ondigitalocean.app/api/units/461187</t>
+      <c r="J9" s="6" t="inlineStr">
+        <is>
+          <t>https://www.shipvault.com/ships/461187, https://shipvaultapi-gjb8c.ondigitalocean.app/api/units/461187, https://www.datocms-assets.com/146580/1763396210-1747916410-igu-world-lng-report-2025.pdf</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
@@ -2279,18 +2330,21 @@
           <t>https://www.igu.org/igu-reports/2025-world-lng-report</t>
         </is>
       </c>
-      <c r="AM9" s="2" t="inlineStr">
-        <is>
-          <t>IGU</t>
-        </is>
-      </c>
+      <c r="AM9" s="2" t="inlineStr"/>
       <c r="AN9" s="2" t="inlineStr"/>
       <c r="AO9" s="2" t="inlineStr"/>
-      <c r="AP9" s="2" t="inlineStr"/>
+      <c r="AP9" s="2" t="inlineStr">
+        <is>
+          <t>IGU</t>
+        </is>
+      </c>
       <c r="AQ9" s="2" t="inlineStr"/>
       <c r="AR9" s="2" t="inlineStr"/>
       <c r="AS9" s="2" t="inlineStr"/>
       <c r="AT9" s="2" t="inlineStr"/>
+      <c r="AU9" s="2" t="inlineStr"/>
+      <c r="AV9" s="2" t="inlineStr"/>
+      <c r="AW9" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2303,7 +2357,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F69"/>
+  <dimension ref="A1:F74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -2315,39 +2369,39 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="6" t="inlineStr">
+      <c r="A1" s="7" t="inlineStr">
         <is>
           <t>Per-cell citation log</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="7" t="inlineStr">
+      <c r="A2" s="8" t="inlineStr">
         <is>
           <t>row_id</t>
         </is>
       </c>
-      <c r="B2" s="7" t="inlineStr">
+      <c r="B2" s="8" t="inlineStr">
         <is>
           <t>field</t>
         </is>
       </c>
-      <c r="C2" s="7" t="inlineStr">
+      <c r="C2" s="8" t="inlineStr">
         <is>
           <t>action</t>
         </is>
       </c>
-      <c r="D2" s="7" t="inlineStr">
+      <c r="D2" s="8" t="inlineStr">
         <is>
           <t>confidence</t>
         </is>
       </c>
-      <c r="E2" s="7" t="inlineStr">
+      <c r="E2" s="8" t="inlineStr">
         <is>
           <t>url</t>
         </is>
       </c>
-      <c r="F2" s="7" t="inlineStr">
+      <c r="F2" s="8" t="inlineStr">
         <is>
           <t>note</t>
         </is>
@@ -2925,7 +2979,7 @@
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>live row 652: value 'China': OK</t>
+          <t>live row 652: value 'China': IGU prints no Shipowner country/area column - the earlier text-search PASS was false (igu_refs, IG §1)</t>
         </is>
       </c>
     </row>
@@ -3958,6 +4012,126 @@
       <c r="F69" s="2" t="inlineStr">
         <is>
           <t>live row 1185: value 'conventional': page does not contain value 'conventional'</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="inlineStr">
+        <is>
+          <t>121</t>
+        </is>
+      </c>
+      <c r="B70" s="2" t="inlineStr">
+        <is>
+          <t>Hull number</t>
+        </is>
+      </c>
+      <c r="C70" s="2" t="inlineStr"/>
+      <c r="D70" s="2" t="inlineStr"/>
+      <c r="E70" s="2" t="inlineStr">
+        <is>
+          <t>https://www.datocms-assets.com/146580/1763396210-1747916410-igu-world-lng-report-2025.pdf</t>
+        </is>
+      </c>
+      <c r="F70" s="2" t="inlineStr">
+        <is>
+          <t>live row 771: IGU 2025 report PDF (stands in for the landing page) prints this hull for the row's IMO - igu_refs.corroborates_cell</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="inlineStr">
+        <is>
+          <t>121</t>
+        </is>
+      </c>
+      <c r="B71" s="2" t="inlineStr">
+        <is>
+          <t>Hull number</t>
+        </is>
+      </c>
+      <c r="C71" s="2" t="inlineStr"/>
+      <c r="D71" s="2" t="inlineStr"/>
+      <c r="E71" s="2" t="inlineStr">
+        <is>
+          <t>https://www.datocms-assets.com/146580/1783403747-igu-world-lng-report-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F71" s="2" t="inlineStr">
+        <is>
+          <t>live row 771: IGU 2026 report PDF (stands in for the landing page) prints this hull for the row's IMO - igu_refs.corroborates_cell</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="inlineStr">
+        <is>
+          <t>226</t>
+        </is>
+      </c>
+      <c r="B72" s="2" t="inlineStr">
+        <is>
+          <t>Hull number</t>
+        </is>
+      </c>
+      <c r="C72" s="2" t="inlineStr"/>
+      <c r="D72" s="2" t="inlineStr"/>
+      <c r="E72" s="2" t="inlineStr">
+        <is>
+          <t>https://www.datocms-assets.com/146580/1763396210-1747916410-igu-world-lng-report-2025.pdf</t>
+        </is>
+      </c>
+      <c r="F72" s="2" t="inlineStr">
+        <is>
+          <t>live row 775: IGU 2025 report PDF (stands in for the landing page) prints this hull for the row's IMO - igu_refs.corroborates_cell</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="inlineStr">
+        <is>
+          <t>226</t>
+        </is>
+      </c>
+      <c r="B73" s="2" t="inlineStr">
+        <is>
+          <t>Hull number</t>
+        </is>
+      </c>
+      <c r="C73" s="2" t="inlineStr"/>
+      <c r="D73" s="2" t="inlineStr"/>
+      <c r="E73" s="2" t="inlineStr">
+        <is>
+          <t>https://www.datocms-assets.com/146580/1783403747-igu-world-lng-report-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F73" s="2" t="inlineStr">
+        <is>
+          <t>live row 775: IGU 2026 report PDF (stands in for the landing page) prints this hull for the row's IMO - igu_refs.corroborates_cell</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="inlineStr">
+        <is>
+          <t>230</t>
+        </is>
+      </c>
+      <c r="B74" s="2" t="inlineStr">
+        <is>
+          <t>Hull number</t>
+        </is>
+      </c>
+      <c r="C74" s="2" t="inlineStr"/>
+      <c r="D74" s="2" t="inlineStr"/>
+      <c r="E74" s="2" t="inlineStr">
+        <is>
+          <t>https://www.datocms-assets.com/146580/1763396210-1747916410-igu-world-lng-report-2025.pdf</t>
+        </is>
+      </c>
+      <c r="F74" s="2" t="inlineStr">
+        <is>
+          <t>live row 776: IGU 2025 report PDF (stands in for the landing page) prints this hull for the row's IMO - igu_refs.corroborates_cell</t>
         </is>
       </c>
     </row>

</xml_diff>